<commit_message>
Add t Stat criterion and report RMSE
Entry and removal can now use a |t| cutoff (default 2.0) or p-values.
The report shows t and p for every step and labels the model's
standard error as RMSE.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UCpSU19FV3N64No8W4EyLE
</commit_message>
<xml_diff>
--- a/excel-stepwise-regression/examples/Stepwise_Example_Output.xlsx
+++ b/excel-stepwise-regression/examples/Stepwise_Example_Output.xlsx
@@ -444,19 +444,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -493,188 +494,169 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P-value to enter</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>0.05</v>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>t Stat</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Observations used</t>
+          <t>|t| to enter</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Rows excluded (blank or non-numeric)</t>
+          <t>Observations used</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Y range</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$A$4:$A$48</t>
-        </is>
+          <t>Rows excluded (blank or non-numeric)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Y range</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$A$4:$A$48</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>X range</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$B$4:$F$48</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Selection steps</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>t Stat</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Terms in model</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>R Square</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>Adjusted R Square</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>Standard Error</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>AIC</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>BIC</t>
         </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Start</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>(intercept only)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>59.50525408962315</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>360.5621471139791</v>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>362.3463367478973</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Entered</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>SENIORITY</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>9.228644748979778e-06</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>1</v>
+          <t>(intercept only)</t>
+        </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.3772382937978863</v>
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.3624106341264074</v>
+        <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>47.51446531724617</v>
+        <v>0</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>341.7241287074199</v>
+        <v>59.50525408962315</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>345.2925079752565</v>
+        <v>360.5621471139791</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>362.3463367478973</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -683,393 +665,449 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>ROW4</t>
+          <t>SENIORITY</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.0007882920406007329</v>
+        <v>5.043959389223088</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>2</v>
+        <v>9.228644748979778e-06</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.5284488333832105</v>
+        <v>1</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.5054463374506841</v>
+        <v>0.3772382937978863</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>41.84677801904596</v>
+        <v>0.3624106341264074</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>331.4861298983806</v>
+        <v>47.51446531724617</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>336.8386988001354</v>
+        <v>341.7241287074199</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>345.2925079752565</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>ROW4</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>-3.625922757261429</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>0.0007882920406007329</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="2" t="n">
+        <v>0.5284488333832105</v>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>0.5054463374506841</v>
+      </c>
+      <c r="I16" s="2" t="n">
+        <v>41.84677801904596</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>331.4861298983806</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>336.8386988001354</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Entered</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>SENIORITY2</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D17" s="2" t="n">
+        <v>-2.268472355328643</v>
+      </c>
+      <c r="E17" s="2" t="n">
         <v>0.02876969615165533</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="F17" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>0.5821986327815938</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="H17" s="2" t="n">
         <v>0.5508635302402132</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="I17" s="2" t="n">
         <v>39.87901974791074</v>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="J17" s="2" t="n">
         <v>328.161184186538</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="K17" s="2" t="n">
         <v>335.297942722211</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Final model</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Regression Statistics</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Multiple R</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n">
-        <v>0.7630194183515868</v>
-      </c>
+      <c r="B20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>R Square</t>
+          <t>Multiple R</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>0.5821986327815938</v>
+        <v>0.7630194183515868</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Adjusted R Square</t>
+          <t>R Square</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>0.5508635302402132</v>
+        <v>0.5821986327815938</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Standard Error</t>
+          <t>Adjusted R Square</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>39.87901974791074</v>
+        <v>0.5508635302402132</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>39.87901974791074</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B25" s="3" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>ANOVA</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>df</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>SS</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E27" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F27" s="5" t="inlineStr">
         <is>
           <t>Significance F</t>
         </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>88644.18772146615</v>
-      </c>
-      <c r="D27" s="2" t="n">
-        <v>29548.06257382205</v>
-      </c>
-      <c r="E27" s="2" t="n">
-        <v>18.57975834011568</v>
-      </c>
-      <c r="F27" s="2" t="n">
-        <v>1.047506197750365e-07</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Residual</t>
+          <t>Regression</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>63613.44864217019</v>
+        <v>88644.18772146615</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>1590.336216054255</v>
+        <v>29548.06257382205</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>18.57975834011568</v>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>1.047506197750365e-07</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t>Residual</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>63613.44864217019</v>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>1590.336216054255</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B30" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C30" s="2" t="n">
         <v>152257.6363636364</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>Term</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>Coefficients</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>Standard Error</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F32" s="5" t="inlineStr">
         <is>
           <t>Lower 95%</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>Upper 95%</t>
         </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Intercept</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>576.8510432717311</v>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>20.34857154869033</v>
-      </c>
-      <c r="D32" s="2" t="n">
-        <v>28.34847851071189</v>
-      </c>
-      <c r="E32" s="2" t="n">
-        <v>4.229859701784347e-28</v>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>535.7250460867867</v>
-      </c>
-      <c r="G32" s="2" t="n">
-        <v>617.9770404566755</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>SENIORITY</t>
+          <t>Intercept</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>18.36699427515806</v>
+        <v>576.8510432717311</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>4.523086573147018</v>
+        <v>20.34857154869033</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>4.06072136319489</v>
+        <v>28.34847851071189</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.0002213651395959524</v>
+        <v>4.229859701784347e-28</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>9.225495313945892</v>
+        <v>535.7250460867867</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>27.50849323637024</v>
+        <v>617.9770404566755</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SENIORITY2</t>
+          <t>SENIORITY</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>-0.4553993767172003</v>
+        <v>18.36699427515806</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>0.2007515655403368</v>
+        <v>4.523086573147018</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>-2.268472355328643</v>
+        <v>4.06072136319489</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.02876969615165533</v>
+        <v>0.0002213651395959524</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>-0.8611334253962319</v>
+        <v>9.225495313945892</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>-0.04966532803816875</v>
+        <v>27.50849323637024</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
+          <t>SENIORITY2</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>-0.4553993767172003</v>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>0.2007515655403368</v>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>-2.268472355328643</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>0.02876969615165533</v>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>-0.8611334253962319</v>
+      </c>
+      <c r="G35" s="2" t="n">
+        <v>-0.04966532803816875</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t>ROW4</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B36" s="2" t="n">
         <v>-157.4795260781477</v>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C36" s="2" t="n">
         <v>41.96728143246101</v>
       </c>
-      <c r="D35" s="2" t="n">
+      <c r="D36" s="2" t="n">
         <v>-3.752435723805065</v>
       </c>
-      <c r="E35" s="2" t="n">
+      <c r="E36" s="2" t="n">
         <v>0.0005559680892052376</v>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="F36" s="2" t="n">
         <v>-242.2985657793521</v>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="G36" s="2" t="n">
         <v>-72.66048637694338</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Variables not in the final model</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>t Stat if entered next</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>P-value if entered next</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>SEX</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>0.5105909682321952</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>SEX</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>-0.6640095613346428</v>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>0.5105909682321952</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
           <t>SEX_SENIOR</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
+      <c r="B41" s="2" t="n">
+        <v>-0.425985245834234</v>
+      </c>
+      <c r="C41" s="2" t="n">
         <v>0.6724604883748416</v>
       </c>
     </row>
@@ -1084,19 +1122,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1133,547 +1172,581 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P-value to remove</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>0.1</v>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>t Stat</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Observations used</t>
+          <t>|t| to remove</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Rows excluded (blank or non-numeric)</t>
+          <t>Observations used</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Y range</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$A$4:$A$48</t>
-        </is>
+          <t>Rows excluded (blank or non-numeric)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Y range</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$A$4:$A$48</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>X range</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$B$4:$F$48</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Selection steps</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>t Stat</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Terms in model</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>R Square</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>Adjusted R Square</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>Standard Error</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>AIC</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>BIC</t>
         </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Start</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>(all candidates)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>0.5876160345682728</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>0.5333549864851509</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>40.6488841857923</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>331.5869291311083</v>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>342.2920669346179</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Removed</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>SEX_SENIOR</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>0.79448446302617</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>4</v>
+          <t>(all candidates)</t>
+        </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>0.5868692213338237</v>
+        <v>5</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>0.5444968337783185</v>
+        <v>0.5876160345682728</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>40.16067596631433</v>
+        <v>0.5333549864851509</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>329.6665395596683</v>
+        <v>40.6488841857923</v>
       </c>
       <c r="J14" s="2" t="n">
-        <v>338.5874877292596</v>
+        <v>331.5869291311083</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>342.2920669346179</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Removed</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>SEX_SENIOR</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>0.2623293697668429</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>0.79448446302617</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" s="2" t="n">
+        <v>0.5868692213338237</v>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>0.5444968337783185</v>
+      </c>
+      <c r="I15" s="2" t="n">
+        <v>40.16067596631433</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>329.6665395596683</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>338.5874877292596</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Removed</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>SEX</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D16" s="2" t="n">
+        <v>-0.6640095613346428</v>
+      </c>
+      <c r="E16" s="2" t="n">
         <v>0.5105909682321952</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="F16" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>0.5821986327815938</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="H16" s="2" t="n">
         <v>0.5508635302402132</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="I16" s="2" t="n">
         <v>39.87901974791074</v>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="J16" s="2" t="n">
         <v>328.161184186538</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="K16" s="2" t="n">
         <v>335.297942722211</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Final model</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Regression Statistics</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Multiple R</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>0.7630194183515868</v>
-      </c>
+      <c r="B19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>R Square</t>
+          <t>Multiple R</t>
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>0.5821986327815938</v>
+        <v>0.7630194183515868</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Adjusted R Square</t>
+          <t>R Square</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>0.5508635302402132</v>
+        <v>0.5821986327815938</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Standard Error</t>
+          <t>Adjusted R Square</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>39.87901974791074</v>
+        <v>0.5508635302402132</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>39.87901974791074</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B24" s="3" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>ANOVA</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>df</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>SS</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E26" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F26" s="5" t="inlineStr">
         <is>
           <t>Significance F</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>88644.18772146615</v>
-      </c>
-      <c r="D26" s="2" t="n">
-        <v>29548.06257382205</v>
-      </c>
-      <c r="E26" s="2" t="n">
-        <v>18.57975834011568</v>
-      </c>
-      <c r="F26" s="2" t="n">
-        <v>1.047506197750365e-07</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Residual</t>
+          <t>Regression</t>
         </is>
       </c>
       <c r="B27" s="2" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>63613.44864217019</v>
+        <v>88644.18772146615</v>
       </c>
       <c r="D27" s="2" t="n">
-        <v>1590.336216054255</v>
+        <v>29548.06257382205</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>18.57975834011568</v>
+      </c>
+      <c r="F27" s="2" t="n">
+        <v>1.047506197750365e-07</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Residual</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>63613.44864217019</v>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>1590.336216054255</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B29" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="C28" s="2" t="n">
+      <c r="C29" s="2" t="n">
         <v>152257.6363636364</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Term</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>Coefficients</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Standard Error</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
-      <c r="E30" s="5" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="F30" s="5" t="inlineStr">
+      <c r="F31" s="5" t="inlineStr">
         <is>
           <t>Lower 95%</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>Upper 95%</t>
         </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Intercept</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>576.8510432717311</v>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>20.34857154869033</v>
-      </c>
-      <c r="D31" s="2" t="n">
-        <v>28.34847851071189</v>
-      </c>
-      <c r="E31" s="2" t="n">
-        <v>4.229859701784347e-28</v>
-      </c>
-      <c r="F31" s="2" t="n">
-        <v>535.7250460867867</v>
-      </c>
-      <c r="G31" s="2" t="n">
-        <v>617.9770404566755</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>SENIORITY</t>
+          <t>Intercept</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>18.36699427515806</v>
+        <v>576.8510432717311</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>4.523086573147018</v>
+        <v>20.34857154869033</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>4.06072136319489</v>
+        <v>28.34847851071189</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.0002213651395959524</v>
+        <v>4.229859701784347e-28</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>9.225495313945892</v>
+        <v>535.7250460867867</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>27.50849323637024</v>
+        <v>617.9770404566755</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>SENIORITY2</t>
+          <t>SENIORITY</t>
         </is>
       </c>
       <c r="B33" s="2" t="n">
-        <v>-0.4553993767172003</v>
+        <v>18.36699427515806</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>0.2007515655403368</v>
+        <v>4.523086573147018</v>
       </c>
       <c r="D33" s="2" t="n">
-        <v>-2.268472355328643</v>
+        <v>4.06072136319489</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.02876969615165533</v>
+        <v>0.0002213651395959524</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>-0.8611334253962319</v>
+        <v>9.225495313945892</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>-0.04966532803816875</v>
+        <v>27.50849323637024</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>SENIORITY2</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>-0.4553993767172003</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>0.2007515655403368</v>
+      </c>
+      <c r="D34" s="2" t="n">
+        <v>-2.268472355328643</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>0.02876969615165533</v>
+      </c>
+      <c r="F34" s="2" t="n">
+        <v>-0.8611334253962319</v>
+      </c>
+      <c r="G34" s="2" t="n">
+        <v>-0.04966532803816875</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>ROW4</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B35" s="2" t="n">
         <v>-157.4795260781477</v>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C35" s="2" t="n">
         <v>41.96728143246101</v>
       </c>
-      <c r="D34" s="2" t="n">
+      <c r="D35" s="2" t="n">
         <v>-3.752435723805065</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E35" s="2" t="n">
         <v>0.0005559680892052376</v>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F35" s="2" t="n">
         <v>-242.2985657793521</v>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="G35" s="2" t="n">
         <v>-72.66048637694338</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>Variables not in the final model</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>t Stat if entered next</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
         <is>
           <t>P-value if entered next</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>SEX</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="n">
-        <v>0.5105909682321952</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t>SEX</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>-0.6640095613346428</v>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>0.5105909682321952</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>SEX_SENIOR</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
+      <c r="B40" s="2" t="n">
+        <v>-0.425985245834234</v>
+      </c>
+      <c r="C40" s="2" t="n">
         <v>0.6724604883748416</v>
       </c>
     </row>
@@ -1688,19 +1761,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1737,198 +1811,179 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>P-value to enter</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>0.05</v>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>t Stat</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>P-value to remove</t>
+          <t>|t| to enter</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Observations used</t>
+          <t>|t| to remove</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Rows excluded (blank or non-numeric)</t>
+          <t>Observations used</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Y range</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$A$4:$A$48</t>
-        </is>
+          <t>Rows excluded (blank or non-numeric)</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Y range</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$A$4:$A$48</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>X range</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$B$4:$F$48</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Selection steps</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>t Stat</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>Terms in model</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>R Square</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="H14" s="5" t="inlineStr">
         <is>
           <t>Adjusted R Square</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
-        <is>
-          <t>Standard Error</t>
-        </is>
-      </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>AIC</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>BIC</t>
         </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Start</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>(intercept only)</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>59.50525408962315</v>
-      </c>
-      <c r="I14" s="2" t="n">
-        <v>360.5621471139791</v>
-      </c>
-      <c r="J14" s="2" t="n">
-        <v>362.3463367478973</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Entered</t>
+          <t>Start</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>SENIORITY</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>9.228644748979778e-06</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>1</v>
+          <t>(intercept only)</t>
+        </is>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.3772382937978863</v>
+        <v>0</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>0.3624106341264074</v>
+        <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>47.51446531724617</v>
+        <v>0</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>341.7241287074199</v>
+        <v>59.50525408962315</v>
       </c>
       <c r="J15" s="2" t="n">
-        <v>345.2925079752565</v>
+        <v>360.5621471139791</v>
+      </c>
+      <c r="K15" s="2" t="n">
+        <v>362.3463367478973</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -1937,393 +1992,449 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>ROW4</t>
+          <t>SENIORITY</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>0.0007882920406007329</v>
+        <v>5.043959389223088</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>2</v>
+        <v>9.228644748979778e-06</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>0.5284488333832105</v>
+        <v>1</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>0.5054463374506841</v>
+        <v>0.3772382937978863</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>41.84677801904596</v>
+        <v>0.3624106341264074</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>331.4861298983806</v>
+        <v>47.51446531724617</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>336.8386988001354</v>
+        <v>341.7241287074199</v>
+      </c>
+      <c r="K16" s="2" t="n">
+        <v>345.2925079752565</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Entered</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>ROW4</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>-3.625922757261429</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>0.0007882920406007329</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="2" t="n">
+        <v>0.5284488333832105</v>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0.5054463374506841</v>
+      </c>
+      <c r="I17" s="2" t="n">
+        <v>41.84677801904596</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>331.4861298983806</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>336.8386988001354</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Entered</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>SENIORITY2</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D18" s="2" t="n">
+        <v>-2.268472355328643</v>
+      </c>
+      <c r="E18" s="2" t="n">
         <v>0.02876969615165533</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="F18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>0.5821986327815938</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="H18" s="2" t="n">
         <v>0.5508635302402132</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="I18" s="2" t="n">
         <v>39.87901974791074</v>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="J18" s="2" t="n">
         <v>328.161184186538</v>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="K18" s="2" t="n">
         <v>335.297942722211</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Final model</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Regression Statistics</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Multiple R</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n">
-        <v>0.7630194183515868</v>
-      </c>
+      <c r="B21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>R Square</t>
+          <t>Multiple R</t>
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>0.5821986327815938</v>
+        <v>0.7630194183515868</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Adjusted R Square</t>
+          <t>R Square</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>0.5508635302402132</v>
+        <v>0.5821986327815938</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Standard Error</t>
+          <t>Adjusted R Square</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>39.87901974791074</v>
+        <v>0.5508635302402132</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>39.87901974791074</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B26" s="3" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>ANOVA</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>df</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>SS</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E28" s="5" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
         <is>
           <t>Significance F</t>
         </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Regression</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>88644.18772146615</v>
-      </c>
-      <c r="D28" s="2" t="n">
-        <v>29548.06257382205</v>
-      </c>
-      <c r="E28" s="2" t="n">
-        <v>18.57975834011568</v>
-      </c>
-      <c r="F28" s="2" t="n">
-        <v>1.047506197750365e-07</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Residual</t>
+          <t>Regression</t>
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>63613.44864217019</v>
+        <v>88644.18772146615</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>1590.336216054255</v>
+        <v>29548.06257382205</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>18.57975834011568</v>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>1.047506197750365e-07</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>Residual</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>63613.44864217019</v>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>1590.336216054255</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B31" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="C30" s="2" t="n">
+      <c r="C31" s="2" t="n">
         <v>152257.6363636364</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>Term</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Coefficients</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>Standard Error</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F33" s="5" t="inlineStr">
         <is>
           <t>Lower 95%</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>Upper 95%</t>
         </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Intercept</t>
-        </is>
-      </c>
-      <c r="B33" s="2" t="n">
-        <v>576.8510432717311</v>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>20.34857154869033</v>
-      </c>
-      <c r="D33" s="2" t="n">
-        <v>28.34847851071189</v>
-      </c>
-      <c r="E33" s="2" t="n">
-        <v>4.229859701784347e-28</v>
-      </c>
-      <c r="F33" s="2" t="n">
-        <v>535.7250460867867</v>
-      </c>
-      <c r="G33" s="2" t="n">
-        <v>617.9770404566755</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>SENIORITY</t>
+          <t>Intercept</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>18.36699427515806</v>
+        <v>576.8510432717311</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>4.523086573147018</v>
+        <v>20.34857154869033</v>
       </c>
       <c r="D34" s="2" t="n">
-        <v>4.06072136319489</v>
+        <v>28.34847851071189</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.0002213651395959524</v>
+        <v>4.229859701784347e-28</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>9.225495313945892</v>
+        <v>535.7250460867867</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>27.50849323637024</v>
+        <v>617.9770404566755</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>SENIORITY2</t>
+          <t>SENIORITY</t>
         </is>
       </c>
       <c r="B35" s="2" t="n">
-        <v>-0.4553993767172003</v>
+        <v>18.36699427515806</v>
       </c>
       <c r="C35" s="2" t="n">
-        <v>0.2007515655403368</v>
+        <v>4.523086573147018</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>-2.268472355328643</v>
+        <v>4.06072136319489</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.02876969615165533</v>
+        <v>0.0002213651395959524</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>-0.8611334253962319</v>
+        <v>9.225495313945892</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>-0.04966532803816875</v>
+        <v>27.50849323637024</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
+          <t>SENIORITY2</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>-0.4553993767172003</v>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>0.2007515655403368</v>
+      </c>
+      <c r="D36" s="2" t="n">
+        <v>-2.268472355328643</v>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>0.02876969615165533</v>
+      </c>
+      <c r="F36" s="2" t="n">
+        <v>-0.8611334253962319</v>
+      </c>
+      <c r="G36" s="2" t="n">
+        <v>-0.04966532803816875</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
           <t>ROW4</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B37" s="2" t="n">
         <v>-157.4795260781477</v>
       </c>
-      <c r="C36" s="2" t="n">
+      <c r="C37" s="2" t="n">
         <v>41.96728143246101</v>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D37" s="2" t="n">
         <v>-3.752435723805065</v>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E37" s="2" t="n">
         <v>0.0005559680892052376</v>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="F37" s="2" t="n">
         <v>-242.2985657793521</v>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="G37" s="2" t="n">
         <v>-72.66048637694338</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>Variables not in the final model</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>t Stat if entered next</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>P-value if entered next</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>SEX</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="n">
-        <v>0.5105909682321952</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
+          <t>SEX</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>-0.6640095613346428</v>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>0.5105909682321952</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
           <t>SEX_SENIOR</t>
         </is>
       </c>
-      <c r="B41" s="2" t="n">
+      <c r="B42" s="2" t="n">
+        <v>-0.425985245834234</v>
+      </c>
+      <c r="C42" s="2" t="n">
         <v>0.6724604883748416</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Style the report in burnt orange with HOUMBA Class of '28 credit
Title bar, section headings and table headers in #BF5700, consistent
number formats, p-values below 0.0001 shown as <0.0001, gridlines off.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UCpSU19FV3N64No8W4EyLE
</commit_message>
<xml_diff>
--- a/excel-stepwise-regression/examples/Stepwise_Example_Output.xlsx
+++ b/excel-stepwise-regression/examples/Stepwise_Example_Output.xlsx
@@ -18,8 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="5">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="[&lt;0.0001]&quot;&lt;0.0001&quot;;0.0000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0000"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,34 +32,63 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00BF5700"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00BF5700"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00595959"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <i val="1"/>
-      <sz val="10"/>
+      <color rgb="00595959"/>
+      <sz val="8"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BF5700"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8E5D6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -64,21 +97,68 @@
       <diagonal/>
     </border>
     <border>
-      <bottom style="thin"/>
+      <bottom style="medium">
+        <color rgb="00BF5700"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00BF5700"/>
+      </top>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,672 +524,708 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Stepwise Regression Output</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+          <t xml:space="preserve">  Stepwise Regression Output</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Built for the HOUMBA Class of '28</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Dependent variable</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>SALARY</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Forward selection</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Criterion</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>|t| to enter</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B8" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Observations used</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B9" s="8" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Rows excluded (blank or non-numeric)</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B10" s="8" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Y range</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$A$4:$A$48</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>X range</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$B$4:$F$48</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Selection steps</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>Terms in model</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G15" s="10" t="inlineStr">
         <is>
           <t>R Square</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H15" s="10" t="inlineStr">
         <is>
           <t>Adjusted R Square</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="J15" s="10" t="inlineStr">
         <is>
           <t>AIC</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>BIC</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>(intercept only)</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G16" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="H16" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="I14" s="2" t="n">
+      <c r="I16" s="13" t="n">
         <v>59.50525408962315</v>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J16" s="13" t="n">
         <v>360.5621471139791</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K16" s="13" t="n">
         <v>362.3463367478973</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
+    <row r="17">
+      <c r="A17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Entered</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>SENIORITY</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D17" s="14" t="n">
         <v>5.043959389223088</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E17" s="15" t="n">
         <v>9.228644748979778e-06</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F17" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G17" s="12" t="n">
         <v>0.3772382937978863</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H17" s="12" t="n">
         <v>0.3624106341264074</v>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="I17" s="13" t="n">
         <v>47.51446531724617</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J17" s="13" t="n">
         <v>341.7241287074199</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K17" s="13" t="n">
         <v>345.2925079752565</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Entered</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>ROW4</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D18" s="14" t="n">
         <v>-3.625922757261429</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E18" s="15" t="n">
         <v>0.0007882920406007329</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F18" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G18" s="12" t="n">
         <v>0.5284488333832105</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="H18" s="12" t="n">
         <v>0.5054463374506841</v>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="I18" s="13" t="n">
         <v>41.84677801904596</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="J18" s="13" t="n">
         <v>331.4861298983806</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K18" s="13" t="n">
         <v>336.8386988001354</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
+    <row r="19">
+      <c r="A19" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Entered</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>SENIORITY2</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D19" s="14" t="n">
         <v>-2.268472355328643</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E19" s="15" t="n">
         <v>0.02876969615165533</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="F19" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G19" s="12" t="n">
         <v>0.5821986327815938</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="H19" s="12" t="n">
         <v>0.5508635302402132</v>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="I19" s="13" t="n">
         <v>39.87901974791074</v>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="J19" s="13" t="n">
         <v>328.161184186538</v>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="K19" s="13" t="n">
         <v>335.297942722211</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Final model</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Regression Statistics</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Multiple R</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B22" s="16" t="n">
         <v>0.7630194183515868</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>R Square</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B23" s="16" t="n">
         <v>0.5821986327815938</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Adjusted R Square</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B24" s="16" t="n">
         <v>0.5508635302402132</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B25" s="17" t="n">
         <v>39.87901974791074</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B26" s="8" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
         <is>
           <t>ANOVA</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>df</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C28" s="10" t="inlineStr">
         <is>
           <t>SS</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D28" s="10" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F28" s="10" t="inlineStr">
         <is>
           <t>Significance F</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B29" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C28" s="2" t="n">
+      <c r="C29" s="13" t="n">
         <v>88644.18772146615</v>
       </c>
-      <c r="D28" s="2" t="n">
+      <c r="D29" s="13" t="n">
         <v>29548.06257382205</v>
       </c>
-      <c r="E28" s="2" t="n">
+      <c r="E29" s="13" t="n">
         <v>18.57975834011568</v>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="F29" s="15" t="n">
         <v>1.047506197750365e-07</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B30" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C30" s="13" t="n">
         <v>63613.44864217019</v>
       </c>
-      <c r="D29" s="2" t="n">
+      <c r="D30" s="13" t="n">
         <v>1590.336216054255</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B31" s="19" t="n">
         <v>43</v>
       </c>
-      <c r="C30" s="2" t="n">
+      <c r="C31" s="20" t="n">
         <v>152257.6363636364</v>
       </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="D31" s="21" t="n"/>
+      <c r="E31" s="21" t="n"/>
+      <c r="F31" s="21" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="9" t="inlineStr">
         <is>
           <t>Term</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Coefficients</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>Standard Error</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D33" s="10" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
-      <c r="E32" s="5" t="inlineStr">
+      <c r="E33" s="10" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="F32" s="5" t="inlineStr">
+      <c r="F33" s="10" t="inlineStr">
         <is>
           <t>Lower 95%</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G33" s="10" t="inlineStr">
         <is>
           <t>Upper 95%</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
+      <c r="B34" s="22" t="n">
         <v>576.8510432717311</v>
       </c>
-      <c r="C33" s="2" t="n">
+      <c r="C34" s="22" t="n">
         <v>20.34857154869033</v>
       </c>
-      <c r="D33" s="2" t="n">
+      <c r="D34" s="14" t="n">
         <v>28.34847851071189</v>
       </c>
-      <c r="E33" s="2" t="n">
+      <c r="E34" s="15" t="n">
         <v>4.229859701784347e-28</v>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="F34" s="22" t="n">
         <v>535.7250460867867</v>
       </c>
-      <c r="G33" s="2" t="n">
+      <c r="G34" s="22" t="n">
         <v>617.9770404566755</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>SENIORITY</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B35" s="22" t="n">
         <v>18.36699427515806</v>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C35" s="22" t="n">
         <v>4.523086573147018</v>
       </c>
-      <c r="D34" s="2" t="n">
+      <c r="D35" s="14" t="n">
         <v>4.06072136319489</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E35" s="15" t="n">
         <v>0.0002213651395959524</v>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F35" s="22" t="n">
         <v>9.225495313945892</v>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="G35" s="22" t="n">
         <v>27.50849323637024</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>SENIORITY2</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B36" s="22" t="n">
         <v>-0.4553993767172003</v>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C36" s="22" t="n">
         <v>0.2007515655403368</v>
       </c>
-      <c r="D35" s="2" t="n">
+      <c r="D36" s="14" t="n">
         <v>-2.268472355328643</v>
       </c>
-      <c r="E35" s="2" t="n">
+      <c r="E36" s="15" t="n">
         <v>0.02876969615165533</v>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="F36" s="22" t="n">
         <v>-0.8611334253962319</v>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="G36" s="22" t="n">
         <v>-0.04966532803816875</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>ROW4</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B37" s="22" t="n">
         <v>-157.4795260781477</v>
       </c>
-      <c r="C36" s="2" t="n">
+      <c r="C37" s="22" t="n">
         <v>41.96728143246101</v>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D37" s="14" t="n">
         <v>-3.752435723805065</v>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E37" s="15" t="n">
         <v>0.0005559680892052376</v>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="F37" s="22" t="n">
         <v>-242.2985657793521</v>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="G37" s="22" t="n">
         <v>-72.66048637694338</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>Variables not in the final model</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>t Stat if entered next</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>P-value if entered next</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>t Stat if added</t>
+        </is>
+      </c>
+      <c r="C40" s="10" t="inlineStr">
+        <is>
+          <t>P-value if added</t>
+        </is>
+      </c>
+      <c r="D40" s="9" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>SEX</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
+      <c r="B41" s="14" t="n">
         <v>-0.6640095613346428</v>
       </c>
-      <c r="C40" s="2" t="n">
+      <c r="C41" s="15" t="n">
         <v>0.5105909682321952</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>SEX_SENIOR</t>
         </is>
       </c>
-      <c r="B41" s="2" t="n">
+      <c r="B42" s="14" t="n">
         <v>-0.425985245834234</v>
       </c>
-      <c r="C41" s="2" t="n">
+      <c r="C42" s="15" t="n">
         <v>0.6724604883748416</v>
       </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="23" t="inlineStr">
+        <is>
+          <t>Stepwise Regression add-in  |  Built for the HOUMBA Class of '28</t>
+        </is>
+      </c>
+      <c r="B44" s="24" t="n"/>
+      <c r="C44" s="24" t="n"/>
+      <c r="D44" s="24" t="n"/>
+      <c r="E44" s="24" t="n"/>
+      <c r="F44" s="24" t="n"/>
+      <c r="G44" s="24" t="n"/>
+      <c r="H44" s="24" t="n"/>
+      <c r="I44" s="24" t="n"/>
+      <c r="J44" s="24" t="n"/>
+      <c r="K44" s="24" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1122,633 +1238,669 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K40"/>
+  <dimension ref="A1:K43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Stepwise Regression Output</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+          <t xml:space="preserve">  Stepwise Regression Output</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Built for the HOUMBA Class of '28</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Dependent variable</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>SALARY</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Backward elimination</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Criterion</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>|t| to remove</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B8" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Observations used</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B9" s="8" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Rows excluded (blank or non-numeric)</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B10" s="8" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Y range</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$A$4:$A$48</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>X range</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$B$4:$F$48</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Selection steps</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D15" s="10" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F15" s="10" t="inlineStr">
         <is>
           <t>Terms in model</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G15" s="10" t="inlineStr">
         <is>
           <t>R Square</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H15" s="10" t="inlineStr">
         <is>
           <t>Adjusted R Square</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I15" s="10" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="J15" s="10" t="inlineStr">
         <is>
           <t>AIC</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>BIC</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
+    <row r="16">
+      <c r="A16" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>(all candidates)</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F16" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G16" s="12" t="n">
         <v>0.5876160345682728</v>
       </c>
-      <c r="H14" s="2" t="n">
+      <c r="H16" s="12" t="n">
         <v>0.5333549864851509</v>
       </c>
-      <c r="I14" s="2" t="n">
+      <c r="I16" s="13" t="n">
         <v>40.6488841857923</v>
       </c>
-      <c r="J14" s="2" t="n">
+      <c r="J16" s="13" t="n">
         <v>331.5869291311083</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K16" s="13" t="n">
         <v>342.2920669346179</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
+    <row r="17">
+      <c r="A17" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Removed</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>SEX_SENIOR</t>
         </is>
       </c>
-      <c r="D15" s="2" t="n">
+      <c r="D17" s="14" t="n">
         <v>0.2623293697668429</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="E17" s="15" t="n">
         <v>0.79448446302617</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F17" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G17" s="12" t="n">
         <v>0.5868692213338237</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H17" s="12" t="n">
         <v>0.5444968337783185</v>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="I17" s="13" t="n">
         <v>40.16067596631433</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J17" s="13" t="n">
         <v>329.6665395596683</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K17" s="13" t="n">
         <v>338.5874877292596</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Removed</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>SEX</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D18" s="14" t="n">
         <v>-0.6640095613346428</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E18" s="15" t="n">
         <v>0.5105909682321952</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F18" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G18" s="12" t="n">
         <v>0.5821986327815938</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="H18" s="12" t="n">
         <v>0.5508635302402132</v>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="I18" s="13" t="n">
         <v>39.87901974791074</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="J18" s="13" t="n">
         <v>328.161184186538</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K18" s="13" t="n">
         <v>335.297942722211</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Final model</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Regression Statistics</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Multiple R</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B21" s="16" t="n">
         <v>0.7630194183515868</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>R Square</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B22" s="16" t="n">
         <v>0.5821986327815938</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Adjusted R Square</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B23" s="16" t="n">
         <v>0.5508635302402132</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B24" s="17" t="n">
         <v>39.87901974791074</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B25" s="8" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
         <is>
           <t>ANOVA</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>df</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="10" t="inlineStr">
         <is>
           <t>SS</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D27" s="10" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="E26" s="5" t="inlineStr">
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="F26" s="5" t="inlineStr">
+      <c r="F27" s="10" t="inlineStr">
         <is>
           <t>Significance F</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B28" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C27" s="2" t="n">
+      <c r="C28" s="13" t="n">
         <v>88644.18772146615</v>
       </c>
-      <c r="D27" s="2" t="n">
+      <c r="D28" s="13" t="n">
         <v>29548.06257382205</v>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E28" s="13" t="n">
         <v>18.57975834011568</v>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="F28" s="15" t="n">
         <v>1.047506197750365e-07</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B29" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="C28" s="2" t="n">
+      <c r="C29" s="13" t="n">
         <v>63613.44864217019</v>
       </c>
-      <c r="D28" s="2" t="n">
+      <c r="D29" s="13" t="n">
         <v>1590.336216054255</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B30" s="19" t="n">
         <v>43</v>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C30" s="20" t="n">
         <v>152257.6363636364</v>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="D30" s="21" t="n"/>
+      <c r="E30" s="21" t="n"/>
+      <c r="F30" s="21" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>Term</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>Coefficients</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C32" s="10" t="inlineStr">
         <is>
           <t>Standard Error</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E32" s="10" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F32" s="10" t="inlineStr">
         <is>
           <t>Lower 95%</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G32" s="10" t="inlineStr">
         <is>
           <t>Upper 95%</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B32" s="2" t="n">
+      <c r="B33" s="22" t="n">
         <v>576.8510432717311</v>
       </c>
-      <c r="C32" s="2" t="n">
+      <c r="C33" s="22" t="n">
         <v>20.34857154869033</v>
       </c>
-      <c r="D32" s="2" t="n">
+      <c r="D33" s="14" t="n">
         <v>28.34847851071189</v>
       </c>
-      <c r="E32" s="2" t="n">
+      <c r="E33" s="15" t="n">
         <v>4.229859701784347e-28</v>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="F33" s="22" t="n">
         <v>535.7250460867867</v>
       </c>
-      <c r="G32" s="2" t="n">
+      <c r="G33" s="22" t="n">
         <v>617.9770404566755</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
         <is>
           <t>SENIORITY</t>
         </is>
       </c>
-      <c r="B33" s="2" t="n">
+      <c r="B34" s="22" t="n">
         <v>18.36699427515806</v>
       </c>
-      <c r="C33" s="2" t="n">
+      <c r="C34" s="22" t="n">
         <v>4.523086573147018</v>
       </c>
-      <c r="D33" s="2" t="n">
+      <c r="D34" s="14" t="n">
         <v>4.06072136319489</v>
       </c>
-      <c r="E33" s="2" t="n">
+      <c r="E34" s="15" t="n">
         <v>0.0002213651395959524</v>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="F34" s="22" t="n">
         <v>9.225495313945892</v>
       </c>
-      <c r="G33" s="2" t="n">
+      <c r="G34" s="22" t="n">
         <v>27.50849323637024</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>SENIORITY2</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B35" s="22" t="n">
         <v>-0.4553993767172003</v>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C35" s="22" t="n">
         <v>0.2007515655403368</v>
       </c>
-      <c r="D34" s="2" t="n">
+      <c r="D35" s="14" t="n">
         <v>-2.268472355328643</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E35" s="15" t="n">
         <v>0.02876969615165533</v>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F35" s="22" t="n">
         <v>-0.8611334253962319</v>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="G35" s="22" t="n">
         <v>-0.04966532803816875</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>ROW4</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B36" s="22" t="n">
         <v>-157.4795260781477</v>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C36" s="22" t="n">
         <v>41.96728143246101</v>
       </c>
-      <c r="D35" s="2" t="n">
+      <c r="D36" s="14" t="n">
         <v>-3.752435723805065</v>
       </c>
-      <c r="E35" s="2" t="n">
+      <c r="E36" s="15" t="n">
         <v>0.0005559680892052376</v>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="F36" s="22" t="n">
         <v>-242.2985657793521</v>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="G36" s="22" t="n">
         <v>-72.66048637694338</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>Variables not in the final model</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B38" s="5" t="inlineStr">
-        <is>
-          <t>t Stat if entered next</t>
-        </is>
-      </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>P-value if entered next</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>t Stat if added</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="inlineStr">
+        <is>
+          <t>P-value if added</t>
+        </is>
+      </c>
+      <c r="D39" s="9" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>SEX</t>
         </is>
       </c>
-      <c r="B39" s="2" t="n">
+      <c r="B40" s="14" t="n">
         <v>-0.6640095613346428</v>
       </c>
-      <c r="C39" s="2" t="n">
+      <c r="C40" s="15" t="n">
         <v>0.5105909682321952</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
         <is>
           <t>SEX_SENIOR</t>
         </is>
       </c>
-      <c r="B40" s="2" t="n">
+      <c r="B41" s="14" t="n">
         <v>-0.425985245834234</v>
       </c>
-      <c r="C40" s="2" t="n">
+      <c r="C41" s="15" t="n">
         <v>0.6724604883748416</v>
       </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="23" t="inlineStr">
+        <is>
+          <t>Stepwise Regression add-in  |  Built for the HOUMBA Class of '28</t>
+        </is>
+      </c>
+      <c r="B43" s="24" t="n"/>
+      <c r="C43" s="24" t="n"/>
+      <c r="D43" s="24" t="n"/>
+      <c r="E43" s="24" t="n"/>
+      <c r="F43" s="24" t="n"/>
+      <c r="G43" s="24" t="n"/>
+      <c r="H43" s="24" t="n"/>
+      <c r="I43" s="24" t="n"/>
+      <c r="J43" s="24" t="n"/>
+      <c r="K43" s="24" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1761,682 +1913,718 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Stepwise Regression Output</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+          <t xml:space="preserve">  Stepwise Regression Output</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Built for the HOUMBA Class of '28</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Settings</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Dependent variable</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>SALARY</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Stepwise</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Criterion</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>|t| to enter</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B8" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>|t| to remove</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B9" s="7" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Observations used</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B10" s="8" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Rows excluded (blank or non-numeric)</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B11" s="8" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Y range</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$A$4:$A$48</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>X range</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>'[Hoyda Discrimination.xlsx]Reg - 5 preds'!$B$4:$F$48</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Selection steps</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Action</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C16" s="9" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D16" s="10" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>Terms in model</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G16" s="10" t="inlineStr">
         <is>
           <t>R Square</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H16" s="10" t="inlineStr">
         <is>
           <t>Adjusted R Square</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I16" s="10" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J16" s="10" t="inlineStr">
         <is>
           <t>AIC</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K16" s="10" t="inlineStr">
         <is>
           <t>BIC</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
+    <row r="17">
+      <c r="A17" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>(intercept only)</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F17" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G17" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="2" t="n">
+      <c r="H17" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="I15" s="2" t="n">
+      <c r="I17" s="13" t="n">
         <v>59.50525408962315</v>
       </c>
-      <c r="J15" s="2" t="n">
+      <c r="J17" s="13" t="n">
         <v>360.5621471139791</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K17" s="13" t="n">
         <v>362.3463367478973</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="n">
+    <row r="18">
+      <c r="A18" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Entered</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>SENIORITY</t>
         </is>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D18" s="14" t="n">
         <v>5.043959389223088</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E18" s="15" t="n">
         <v>9.228644748979778e-06</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F18" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G18" s="12" t="n">
         <v>0.3772382937978863</v>
       </c>
-      <c r="H16" s="2" t="n">
+      <c r="H18" s="12" t="n">
         <v>0.3624106341264074</v>
       </c>
-      <c r="I16" s="2" t="n">
+      <c r="I18" s="13" t="n">
         <v>47.51446531724617</v>
       </c>
-      <c r="J16" s="2" t="n">
+      <c r="J18" s="13" t="n">
         <v>341.7241287074199</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K18" s="13" t="n">
         <v>345.2925079752565</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="n">
+    <row r="19">
+      <c r="A19" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>Entered</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>ROW4</t>
         </is>
       </c>
-      <c r="D17" s="2" t="n">
+      <c r="D19" s="14" t="n">
         <v>-3.625922757261429</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="E19" s="15" t="n">
         <v>0.0007882920406007329</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="F19" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G19" s="12" t="n">
         <v>0.5284488333832105</v>
       </c>
-      <c r="H17" s="2" t="n">
+      <c r="H19" s="12" t="n">
         <v>0.5054463374506841</v>
       </c>
-      <c r="I17" s="2" t="n">
+      <c r="I19" s="13" t="n">
         <v>41.84677801904596</v>
       </c>
-      <c r="J17" s="2" t="n">
+      <c r="J19" s="13" t="n">
         <v>331.4861298983806</v>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="K19" s="13" t="n">
         <v>336.8386988001354</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="n">
+    <row r="20">
+      <c r="A20" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Entered</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>SENIORITY2</t>
         </is>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D20" s="14" t="n">
         <v>-2.268472355328643</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E20" s="15" t="n">
         <v>0.02876969615165533</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="F20" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G20" s="12" t="n">
         <v>0.5821986327815938</v>
       </c>
-      <c r="H18" s="2" t="n">
+      <c r="H20" s="12" t="n">
         <v>0.5508635302402132</v>
       </c>
-      <c r="I18" s="2" t="n">
+      <c r="I20" s="13" t="n">
         <v>39.87901974791074</v>
       </c>
-      <c r="J18" s="2" t="n">
+      <c r="J20" s="13" t="n">
         <v>328.161184186538</v>
       </c>
-      <c r="K18" s="2" t="n">
+      <c r="K20" s="13" t="n">
         <v>335.297942722211</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>Final model</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Regression Statistics</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Multiple R</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B23" s="16" t="n">
         <v>0.7630194183515868</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>R Square</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B24" s="16" t="n">
         <v>0.5821986327815938</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Adjusted R Square</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B25" s="16" t="n">
         <v>0.5508635302402132</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B26" s="17" t="n">
         <v>39.87901974791074</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Observations</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B27" s="8" t="n">
         <v>44</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>ANOVA</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>df</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="10" t="inlineStr">
         <is>
           <t>SS</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D29" s="10" t="inlineStr">
         <is>
           <t>MS</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F29" s="10" t="inlineStr">
         <is>
           <t>Significance F</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B30" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C29" s="2" t="n">
+      <c r="C30" s="13" t="n">
         <v>88644.18772146615</v>
       </c>
-      <c r="D29" s="2" t="n">
+      <c r="D30" s="13" t="n">
         <v>29548.06257382205</v>
       </c>
-      <c r="E29" s="2" t="n">
+      <c r="E30" s="13" t="n">
         <v>18.57975834011568</v>
       </c>
-      <c r="F29" s="2" t="n">
+      <c r="F30" s="15" t="n">
         <v>1.047506197750365e-07</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Residual</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B31" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="C30" s="2" t="n">
+      <c r="C31" s="13" t="n">
         <v>63613.44864217019</v>
       </c>
-      <c r="D30" s="2" t="n">
+      <c r="D31" s="13" t="n">
         <v>1590.336216054255</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="18" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n">
+      <c r="B32" s="19" t="n">
         <v>43</v>
       </c>
-      <c r="C31" s="2" t="n">
+      <c r="C32" s="20" t="n">
         <v>152257.6363636364</v>
       </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="D32" s="21" t="n"/>
+      <c r="E32" s="21" t="n"/>
+      <c r="F32" s="21" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>Term</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B34" s="10" t="inlineStr">
         <is>
           <t>Coefficients</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>Standard Error</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D34" s="10" t="inlineStr">
         <is>
           <t>t Stat</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E34" s="10" t="inlineStr">
         <is>
           <t>P-value</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F34" s="10" t="inlineStr">
         <is>
           <t>Lower 95%</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G34" s="10" t="inlineStr">
         <is>
           <t>Upper 95%</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B34" s="2" t="n">
+      <c r="B35" s="22" t="n">
         <v>576.8510432717311</v>
       </c>
-      <c r="C34" s="2" t="n">
+      <c r="C35" s="22" t="n">
         <v>20.34857154869033</v>
       </c>
-      <c r="D34" s="2" t="n">
+      <c r="D35" s="14" t="n">
         <v>28.34847851071189</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="E35" s="15" t="n">
         <v>4.229859701784347e-28</v>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F35" s="22" t="n">
         <v>535.7250460867867</v>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="G35" s="22" t="n">
         <v>617.9770404566755</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
         <is>
           <t>SENIORITY</t>
         </is>
       </c>
-      <c r="B35" s="2" t="n">
+      <c r="B36" s="22" t="n">
         <v>18.36699427515806</v>
       </c>
-      <c r="C35" s="2" t="n">
+      <c r="C36" s="22" t="n">
         <v>4.523086573147018</v>
       </c>
-      <c r="D35" s="2" t="n">
+      <c r="D36" s="14" t="n">
         <v>4.06072136319489</v>
       </c>
-      <c r="E35" s="2" t="n">
+      <c r="E36" s="15" t="n">
         <v>0.0002213651395959524</v>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="F36" s="22" t="n">
         <v>9.225495313945892</v>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="G36" s="22" t="n">
         <v>27.50849323637024</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>SENIORITY2</t>
         </is>
       </c>
-      <c r="B36" s="2" t="n">
+      <c r="B37" s="22" t="n">
         <v>-0.4553993767172003</v>
       </c>
-      <c r="C36" s="2" t="n">
+      <c r="C37" s="22" t="n">
         <v>0.2007515655403368</v>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D37" s="14" t="n">
         <v>-2.268472355328643</v>
       </c>
-      <c r="E36" s="2" t="n">
+      <c r="E37" s="15" t="n">
         <v>0.02876969615165533</v>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="F37" s="22" t="n">
         <v>-0.8611334253962319</v>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="G37" s="22" t="n">
         <v>-0.04966532803816875</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>ROW4</t>
         </is>
       </c>
-      <c r="B37" s="2" t="n">
+      <c r="B38" s="22" t="n">
         <v>-157.4795260781477</v>
       </c>
-      <c r="C37" s="2" t="n">
+      <c r="C38" s="22" t="n">
         <v>41.96728143246101</v>
       </c>
-      <c r="D37" s="2" t="n">
+      <c r="D38" s="14" t="n">
         <v>-3.752435723805065</v>
       </c>
-      <c r="E37" s="2" t="n">
+      <c r="E38" s="15" t="n">
         <v>0.0005559680892052376</v>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="F38" s="22" t="n">
         <v>-242.2985657793521</v>
       </c>
-      <c r="G37" s="2" t="n">
+      <c r="G38" s="22" t="n">
         <v>-72.66048637694338</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>Variables not in the final model</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
         <is>
           <t>Variable</t>
         </is>
       </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>t Stat if entered next</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>P-value if entered next</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>t Stat if added</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="inlineStr">
+        <is>
+          <t>P-value if added</t>
+        </is>
+      </c>
+      <c r="D41" s="9" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
         <is>
           <t>SEX</t>
         </is>
       </c>
-      <c r="B41" s="2" t="n">
+      <c r="B42" s="14" t="n">
         <v>-0.6640095613346428</v>
       </c>
-      <c r="C41" s="2" t="n">
+      <c r="C42" s="15" t="n">
         <v>0.5105909682321952</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
         <is>
           <t>SEX_SENIOR</t>
         </is>
       </c>
-      <c r="B42" s="2" t="n">
+      <c r="B43" s="14" t="n">
         <v>-0.425985245834234</v>
       </c>
-      <c r="C42" s="2" t="n">
+      <c r="C43" s="15" t="n">
         <v>0.6724604883748416</v>
       </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="23" t="inlineStr">
+        <is>
+          <t>Stepwise Regression add-in  |  Built for the HOUMBA Class of '28</t>
+        </is>
+      </c>
+      <c r="B45" s="24" t="n"/>
+      <c r="C45" s="24" t="n"/>
+      <c r="D45" s="24" t="n"/>
+      <c r="E45" s="24" t="n"/>
+      <c r="F45" s="24" t="n"/>
+      <c r="G45" s="24" t="n"/>
+      <c r="H45" s="24" t="n"/>
+      <c r="I45" s="24" t="n"/>
+      <c r="J45" s="24" t="n"/>
+      <c r="K45" s="24" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>